<commit_message>
fix order tracking security system
</commit_message>
<xml_diff>
--- a/trial 1.xlsx
+++ b/trial 1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mohamed adel work\cesar-store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6864C012-536E-4959-B711-1BE0C9BBC0B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B9F3BDA-F240-4349-96AC-EA1F43C2F11D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{791D22A4-40A8-4DDB-9123-A17DB6BCCBDF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="31">
   <si>
     <t>additives-fluids</t>
   </si>
@@ -126,6 +126,9 @@
   </si>
   <si>
     <t>/products/fluids/1.jpg</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
 </sst>
 </file>
@@ -661,6 +664,9 @@
       <c r="H2" t="s">
         <v>1</v>
       </c>
+      <c r="I2" t="s">
+        <v>30</v>
+      </c>
       <c r="J2" t="b">
         <v>1</v>
       </c>
@@ -690,6 +696,9 @@
       <c r="H3" s="1" t="s">
         <v>29</v>
       </c>
+      <c r="I3" t="s">
+        <v>30</v>
+      </c>
       <c r="J3" t="b">
         <v>1</v>
       </c>
@@ -719,6 +728,9 @@
       <c r="H4" t="s">
         <v>1</v>
       </c>
+      <c r="I4" t="s">
+        <v>30</v>
+      </c>
       <c r="J4" t="b">
         <v>1</v>
       </c>
@@ -748,6 +760,9 @@
       <c r="H5" t="s">
         <v>1</v>
       </c>
+      <c r="I5" t="s">
+        <v>30</v>
+      </c>
       <c r="J5" t="b">
         <v>1</v>
       </c>
@@ -777,6 +792,9 @@
       <c r="H6" t="s">
         <v>1</v>
       </c>
+      <c r="I6" t="s">
+        <v>30</v>
+      </c>
       <c r="J6" t="b">
         <v>1</v>
       </c>
@@ -805,6 +823,9 @@
       </c>
       <c r="H7" t="s">
         <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>30</v>
       </c>
       <c r="J7" t="b">
         <v>1</v>

</xml_diff>